<commit_message>
Upgrade models with health insurance covariate
</commit_message>
<xml_diff>
--- a/03_Output/Models/Tables/Tab_Exposure_PO.xlsx
+++ b/03_Output/Models/Tables/Tab_Exposure_PO.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0.877 (0.755-1.018)</t>
+          <t>0.876 (0.754-1.017)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>0.875 (0.763-1.004)</t>
+          <t>0.874 (0.761-1.003)</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -475,7 +475,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>0.998 (0.996-0.999)</t>
+          <t>0.998 (0.997-0.999)</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -485,7 +485,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0.848 (0.736-0.978)</t>
+          <t>0.850 (0.737-0.979)</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -495,7 +495,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>0.875 (0.796-0.962)</t>
+          <t>0.877 (0.798-0.963)</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1.007 (1.001-1.013)</t>
+          <t>1.006 (1.000-1.013)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -527,7 +527,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1.583 (1.083-2.313)</t>
+          <t>1.539 (1.052-2.251)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -537,7 +537,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1.531 (1.093-2.143)</t>
+          <t>1.492 (1.065-2.089)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -557,7 +557,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1.228 (0.900-1.677)</t>
+          <t>1.226 (0.898-1.674)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -567,7 +567,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>1.142 (0.956-1.365)</t>
+          <t>1.152 (0.964-1.376)</t>
         </is>
       </c>
     </row>
@@ -599,7 +599,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.809 (0.654-1.001)</t>
+          <t>0.813 (0.657-1.006)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -609,7 +609,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>0.798 (0.653-0.976)</t>
+          <t>0.802 (0.656-0.981)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0.808 (0.660-0.989)</t>
+          <t>0.811 (0.662-0.993)</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -639,7 +639,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0.841 (0.731-0.967)</t>
+          <t>0.842 (0.732-0.969)</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1.001 (0.995-1.007)</t>
+          <t>1.000 (0.994-1.006)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1.135 (0.781-1.651)</t>
+          <t>1.089 (0.748-1.585)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1.096 (0.791-1.520)</t>
+          <t>1.057 (0.762-1.466)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -701,7 +701,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0.878 (0.649-1.187)</t>
+          <t>0.867 (0.641-1.172)</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -711,7 +711,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>0.873 (0.738-1.032)</t>
+          <t>0.874 (0.739-1.034)</t>
         </is>
       </c>
     </row>
@@ -733,7 +733,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1.004 (0.996-1.013)</t>
+          <t>1.004 (0.995-1.012)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1.474 (0.854-2.544)</t>
+          <t>1.444 (0.836-2.492)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1.377 (0.835-2.271)</t>
+          <t>1.345 (0.815-2.219)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -763,7 +763,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>0.997 (0.994-1.001)</t>
+          <t>0.998 (0.994-1.001)</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -773,7 +773,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0.961 (0.616-1.499)</t>
+          <t>0.967 (0.620-1.508)</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>0.883 (0.686-1.137)</t>
+          <t>0.896 (0.696-1.154)</t>
         </is>
       </c>
     </row>
@@ -815,7 +815,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0.963 (0.668-1.387)</t>
+          <t>0.967 (0.671-1.392)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -825,7 +825,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1.007 (0.725-1.398)</t>
+          <t>1.010 (0.728-1.401)</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0.857 (0.602-1.221)</t>
+          <t>0.863 (0.606-1.229)</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -855,7 +855,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>0.894 (0.708-1.128)</t>
+          <t>0.899 (0.713-1.133)</t>
         </is>
       </c>
     </row>
@@ -877,7 +877,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.000 (0.986-1.015)</t>
+          <t>1.000 (0.985-1.015)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0.968 (0.389-2.406)</t>
+          <t>0.942 (0.379-2.343)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -897,7 +897,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1.022 (0.454-2.301)</t>
+          <t>0.999 (0.444-2.248)</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>0.995 (0.989-1.002)</t>
+          <t>0.996 (0.989-1.002)</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -917,7 +917,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0.671 (0.312-1.441)</t>
+          <t>0.666 (0.310-1.432)</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>0.729 (0.461-1.151)</t>
+          <t>0.734 (0.465-1.159)</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.999 (0.990-1.007)</t>
+          <t>0.999 (0.990-1.008)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0.963 (0.572-1.621)</t>
+          <t>0.978 (0.581-1.646)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>0.955 (0.586-1.556)</t>
+          <t>0.967 (0.594-1.575)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -989,7 +989,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0.942 (0.570-1.557)</t>
+          <t>0.956 (0.578-1.581)</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -999,7 +999,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>0.952 (0.671-1.349)</t>
+          <t>0.959 (0.676-1.360)</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.996 (0.982-1.010)</t>
+          <t>0.996 (0.981-1.010)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0.734 (0.293-1.841)</t>
+          <t>0.714 (0.284-1.794)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1041,7 +1041,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>0.795 (0.355-1.781)</t>
+          <t>0.778 (0.347-1.744)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1061,7 +1061,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0.456 (0.212-0.982)</t>
+          <t>0.453 (0.210-0.977)</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>0.558 (0.357-0.872)</t>
+          <t>0.562 (0.360-0.880)</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1.831 (0.479-7.006)</t>
+          <t>1.833 (0.480-7.002)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1.866 (0.548-6.351)</t>
+          <t>1.855 (0.546-6.300)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>0.991 (0.983-1.000)</t>
+          <t>0.992 (0.983-1.000)</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0.774 (0.256-2.339)</t>
+          <t>0.789 (0.262-2.379)</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>0.630 (0.331-1.201)</t>
+          <t>0.646 (0.340-1.230)</t>
         </is>
       </c>
     </row>
@@ -1175,7 +1175,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0.925 (0.552-1.548)</t>
+          <t>0.928 (0.554-1.554)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>0.978 (0.613-1.562)</t>
+          <t>0.981 (0.614-1.566)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>1.045 (0.648-1.685)</t>
+          <t>1.050 (0.651-1.693)</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>1.064 (0.786-1.441)</t>
+          <t>1.067 (0.789-1.444)</t>
         </is>
       </c>
     </row>
@@ -1237,7 +1237,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1.009 (0.988-1.030)</t>
+          <t>1.008 (0.987-1.029)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1247,7 +1247,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1.430 (0.398-5.141)</t>
+          <t>1.332 (0.371-4.784)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1.423 (0.461-4.390)</t>
+          <t>1.336 (0.434-4.116)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>1.002 (0.994-1.011)</t>
+          <t>1.003 (0.994-1.011)</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>1.343 (0.461-3.917)</t>
+          <t>1.312 (0.450-3.821)</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>1.110 (0.606-2.034)</t>
+          <t>1.113 (0.608-2.037)</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1319,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.581 (0.273-1.236)</t>
+          <t>0.593 (0.279-1.258)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1329,7 +1329,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>0.575 (0.282-1.170)</t>
+          <t>0.586 (0.289-1.190)</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1349,7 +1349,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0.678 (0.333-1.382)</t>
+          <t>0.686 (0.337-1.398)</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>0.801 (0.493-1.301)</t>
+          <t>0.805 (0.496-1.308)</t>
         </is>
       </c>
     </row>
@@ -1381,7 +1381,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0.999 (0.979-1.019)</t>
+          <t>0.998 (0.978-1.018)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1391,7 +1391,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.785 (0.217-2.837)</t>
+          <t>0.725 (0.200-2.621)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>0.824 (0.267-2.539)</t>
+          <t>0.769 (0.249-2.370)</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1421,7 +1421,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0.863 (0.301-2.479)</t>
+          <t>0.835 (0.291-2.397)</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>0.886 (0.494-1.588)</t>
+          <t>0.882 (0.492-1.580)</t>
         </is>
       </c>
     </row>
@@ -1453,7 +1453,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.994 (0.967-1.023)</t>
+          <t>0.994 (0.967-1.022)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>0.594 (0.096-3.697)</t>
+          <t>0.578 (0.093-3.587)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>0.568 (0.107-3.022)</t>
+          <t>0.552 (0.104-2.926)</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0.793 (0.174-3.612)</t>
+          <t>0.794 (0.175-3.598)</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>0.814 (0.342-1.936)</t>
+          <t>0.827 (0.349-1.963)</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>0.843 (0.706-1.005)</t>
+          <t>0.840 (0.704-1.002)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1545,7 +1545,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>0.830 (0.705-0.977)</t>
+          <t>0.827 (0.703-0.974)</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0.824 (0.697-0.973)</t>
+          <t>0.823 (0.696-0.973)</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>0.849 (0.759-0.950)</t>
+          <t>0.850 (0.759-0.950)</t>
         </is>
       </c>
     </row>
@@ -1597,7 +1597,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1.009 (1.001-1.016)</t>
+          <t>1.008 (1.001-1.015)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>1.877 (1.201-2.934)</t>
+          <t>1.840 (1.177-2.878)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>1.762 (1.187-2.616)</t>
+          <t>1.729 (1.164-2.568)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1637,7 +1637,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>1.574 (1.095-2.263)</t>
+          <t>1.579 (1.098-2.271)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1647,7 +1647,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>1.302 (1.059-1.602)</t>
+          <t>1.314 (1.068-1.616)</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1679,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>0.748 (0.582-0.961)</t>
+          <t>0.747 (0.581-0.960)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1689,7 +1689,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>0.743 (0.586-0.943)</t>
+          <t>0.743 (0.586-0.942)</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1709,7 +1709,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0.733 (0.578-0.930)</t>
+          <t>0.732 (0.577-0.930)</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>0.790 (0.670-0.931)</t>
+          <t>0.788 (0.668-0.929)</t>
         </is>
       </c>
     </row>
@@ -1751,7 +1751,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>1.316 (0.848-2.043)</t>
+          <t>1.271 (0.818-1.974)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1761,7 +1761,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1.228 (0.837-1.801)</t>
+          <t>1.189 (0.811-1.745)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1781,7 +1781,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>1.113 (0.784-1.579)</t>
+          <t>1.102 (0.776-1.565)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1791,7 +1791,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>0.985 (0.812-1.194)</t>
+          <t>0.986 (0.813-1.196)</t>
         </is>
       </c>
     </row>
@@ -1813,7 +1813,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1.002 (0.992-1.012)</t>
+          <t>1.001 (0.991-1.011)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>1.271 (0.666-2.424)</t>
+          <t>1.235 (0.647-2.358)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>1.197 (0.662-2.167)</t>
+          <t>1.164 (0.643-2.106)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0.979 (0.580-1.650)</t>
+          <t>0.980 (0.581-1.653)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1863,7 +1863,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>0.914 (0.679-1.229)</t>
+          <t>0.922 (0.686-1.240)</t>
         </is>
       </c>
     </row>
@@ -1895,7 +1895,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>0.894 (0.757-1.056)</t>
+          <t>0.897 (0.759-1.059)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>0.894 (0.768-1.042)</t>
+          <t>0.896 (0.769-1.044)</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1925,7 +1925,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0.880 (0.752-1.031)</t>
+          <t>0.884 (0.755-1.035)</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -1935,7 +1935,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>0.890 (0.802-0.988)</t>
+          <t>0.893 (0.804-0.991)</t>
         </is>
       </c>
     </row>
@@ -1957,7 +1957,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.002 (0.995-1.009)</t>
+          <t>1.001 (0.994-1.008)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1967,7 +1967,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.062 (0.694-1.625)</t>
+          <t>1.026 (0.670-1.571)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1977,7 +1977,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1.087 (0.745-1.586)</t>
+          <t>1.053 (0.722-1.537)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1997,7 +1997,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.027 (0.724-1.457)</t>
+          <t>1.016 (0.716-1.442)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2007,7 +2007,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>0.963 (0.786-1.180)</t>
+          <t>0.967 (0.789-1.185)</t>
         </is>
       </c>
     </row>
@@ -2039,7 +2039,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>0.860 (0.678-1.090)</t>
+          <t>0.870 (0.687-1.103)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2049,7 +2049,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>0.843 (0.674-1.054)</t>
+          <t>0.853 (0.682-1.066)</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0.855 (0.683-1.071)</t>
+          <t>0.864 (0.689-1.082)</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>0.873 (0.747-1.020)</t>
+          <t>0.877 (0.750-1.025)</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>1.000 (0.993-1.006)</t>
+          <t>0.999 (0.993-1.006)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2111,7 +2111,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>0.942 (0.622-1.427)</t>
+          <t>0.903 (0.595-1.368)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2121,7 +2121,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>0.965 (0.672-1.387)</t>
+          <t>0.930 (0.647-1.336)</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0.889 (0.635-1.243)</t>
+          <t>0.874 (0.624-1.222)</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2151,7 +2151,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>0.860 (0.713-1.036)</t>
+          <t>0.860 (0.713-1.037)</t>
         </is>
       </c>
     </row>
@@ -2173,7 +2173,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>0.999 (0.990-1.009)</t>
+          <t>0.999 (0.990-1.008)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>1.016 (0.552-1.871)</t>
+          <t>1.011 (0.549-1.863)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>0.979 (0.560-1.711)</t>
+          <t>0.971 (0.555-1.697)</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2213,7 +2213,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0.909 (0.553-1.494)</t>
+          <t>0.918 (0.559-1.509)</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -2223,7 +2223,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>0.772 (0.581-1.027)</t>
+          <t>0.786 (0.591-1.044)</t>
         </is>
       </c>
     </row>
@@ -2255,7 +2255,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>0.912 (0.672-1.237)</t>
+          <t>0.914 (0.674-1.239)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>0.900 (0.681-1.190)</t>
+          <t>0.901 (0.682-1.192)</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2285,7 +2285,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0.936 (0.703-1.245)</t>
+          <t>0.938 (0.705-1.247)</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>0.932 (0.773-1.125)</t>
+          <t>0.934 (0.774-1.126)</t>
         </is>
       </c>
     </row>
@@ -2317,7 +2317,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>0.993 (0.980-1.006)</t>
+          <t>0.992 (0.980-1.005)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2327,7 +2327,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>0.537 (0.240-1.202)</t>
+          <t>0.529 (0.236-1.183)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>0.603 (0.294-1.237)</t>
+          <t>0.594 (0.290-1.218)</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2357,7 +2357,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0.883 (0.458-1.700)</t>
+          <t>0.878 (0.456-1.691)</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>0.848 (0.575-1.250)</t>
+          <t>0.850 (0.576-1.253)</t>
         </is>
       </c>
     </row>
@@ -2399,7 +2399,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>0.889 (0.573-1.380)</t>
+          <t>0.894 (0.576-1.387)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2409,7 +2409,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>0.868 (0.572-1.315)</t>
+          <t>0.872 (0.576-1.322)</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2429,7 +2429,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0.872 (0.577-1.320)</t>
+          <t>0.877 (0.579-1.326)</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>0.895 (0.672-1.193)</t>
+          <t>0.897 (0.673-1.195)</t>
         </is>
       </c>
     </row>
@@ -2461,7 +2461,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>0.997 (0.985-1.008)</t>
+          <t>0.996 (0.985-1.008)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2471,7 +2471,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>0.673 (0.316-1.435)</t>
+          <t>0.658 (0.309-1.404)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>0.756 (0.391-1.460)</t>
+          <t>0.741 (0.384-1.433)</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2501,7 +2501,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>1.056 (0.576-1.935)</t>
+          <t>1.046 (0.570-1.917)</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2511,7 +2511,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>0.991 (0.710-1.384)</t>
+          <t>0.990 (0.709-1.382)</t>
         </is>
       </c>
     </row>
@@ -2543,7 +2543,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>0.346 (0.109-1.103)</t>
+          <t>0.345 (0.108-1.100)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>0.362 (0.126-1.041)</t>
+          <t>0.361 (0.125-1.037)</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2573,7 +2573,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0.714 (0.282-1.805)</t>
+          <t>0.718 (0.284-1.813)</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>0.700 (0.411-1.192)</t>
+          <t>0.705 (0.414-1.201)</t>
         </is>
       </c>
     </row>
@@ -2625,7 +2625,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1.087 (0.965-1.224)</t>
+          <t>1.088 (0.966-1.224)</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2645,7 +2645,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>1.126 (0.996-1.272)</t>
+          <t>1.126 (0.996-1.273)</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>1.041 (0.962-1.127)</t>
+          <t>1.042 (0.962-1.127)</t>
         </is>
       </c>
     </row>
@@ -2687,7 +2687,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>1.124 (0.791-1.596)</t>
+          <t>1.127 (0.793-1.602)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2697,7 +2697,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1.076 (0.787-1.472)</t>
+          <t>1.079 (0.788-1.475)</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2717,7 +2717,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>1.230 (0.926-1.635)</t>
+          <t>1.231 (0.926-1.636)</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>0.933 (0.791-1.102)</t>
+          <t>0.934 (0.791-1.103)</t>
         </is>
       </c>
     </row>
@@ -2759,7 +2759,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>1.105 (0.913-1.339)</t>
+          <t>1.106 (0.913-1.340)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2769,7 +2769,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1.107 (0.924-1.325)</t>
+          <t>1.107 (0.925-1.326)</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2789,7 +2789,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>1.094 (0.913-1.310)</t>
+          <t>1.095 (0.914-1.311)</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2799,7 +2799,7 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>1.074 (0.950-1.216)</t>
+          <t>1.075 (0.950-1.216)</t>
         </is>
       </c>
     </row>
@@ -2831,7 +2831,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>1.212 (0.863-1.704)</t>
+          <t>1.218 (0.866-1.712)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>1.163 (0.865-1.564)</t>
+          <t>1.167 (0.868-1.570)</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2861,7 +2861,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>1.322 (1.009-1.733)</t>
+          <t>1.324 (1.010-1.736)</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>0.979 (0.844-1.136)</t>
+          <t>0.980 (0.845-1.137)</t>
         </is>
       </c>
     </row>
@@ -2893,7 +2893,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>1.006 (0.998-1.014)</t>
+          <t>1.006 (0.999-1.014)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>1.562 (0.942-2.592)</t>
+          <t>1.572 (0.948-2.610)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2913,7 +2913,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>1.481 (0.932-2.352)</t>
+          <t>1.490 (0.938-2.367)</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>1.749 (1.167-2.622)</t>
+          <t>1.754 (1.170-2.630)</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2943,7 +2943,7 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>1.045 (0.832-1.313)</t>
+          <t>1.047 (0.834-1.316)</t>
         </is>
       </c>
     </row>
@@ -3047,7 +3047,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.998 (0.996-1.000)</t>
+          <t>0.998 (0.995-1.000)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -3057,7 +3057,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0.883 (0.767-1.017)</t>
+          <t>0.883 (0.766-1.017)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -3067,7 +3067,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>0.881 (0.773-1.004)</t>
+          <t>0.881 (0.773-1.003)</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0.855 (0.747-0.978)</t>
+          <t>0.856 (0.748-0.980)</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -3097,7 +3097,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>0.880 (0.804-0.962)</t>
+          <t>0.881 (0.806-0.964)</t>
         </is>
       </c>
     </row>
@@ -3129,7 +3129,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1.604 (1.112-2.314)</t>
+          <t>1.559 (1.080-2.249)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -3139,7 +3139,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1.550 (1.120-2.145)</t>
+          <t>1.511 (1.092-2.092)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -3159,7 +3159,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1.230 (0.912-1.659)</t>
+          <t>1.226 (0.909-1.653)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -3169,7 +3169,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>1.140 (0.961-1.353)</t>
+          <t>1.149 (0.969-1.363)</t>
         </is>
       </c>
     </row>
@@ -3201,7 +3201,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.809 (0.660-0.991)</t>
+          <t>0.812 (0.663-0.995)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -3211,7 +3211,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>0.798 (0.658-0.967)</t>
+          <t>0.800 (0.660-0.970)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -3231,7 +3231,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0.810 (0.668-0.982)</t>
+          <t>0.812 (0.670-0.985)</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1.001 (0.995-1.007)</t>
+          <t>1.000 (0.995-1.006)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -3273,7 +3273,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1.140 (0.797-1.631)</t>
+          <t>1.096 (0.765-1.568)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1.098 (0.804-1.501)</t>
+          <t>1.061 (0.776-1.451)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -3303,7 +3303,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0.873 (0.655-1.164)</t>
+          <t>0.862 (0.647-1.149)</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -3313,7 +3313,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>0.868 (0.740-1.018)</t>
+          <t>0.870 (0.742-1.020)</t>
         </is>
       </c>
     </row>
@@ -3335,7 +3335,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1.005 (0.996-1.013)</t>
+          <t>1.004 (0.996-1.012)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -3345,7 +3345,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1.513 (0.891-2.570)</t>
+          <t>1.473 (0.867-2.503)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1.406 (0.865-2.285)</t>
+          <t>1.367 (0.841-2.222)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -3365,7 +3365,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>0.997 (0.994-1.001)</t>
+          <t>0.998 (0.995-1.001)</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -3375,7 +3375,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0.963 (0.628-1.477)</t>
+          <t>0.964 (0.629-1.478)</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -3385,7 +3385,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>0.879 (0.690-1.120)</t>
+          <t>0.890 (0.698-1.133)</t>
         </is>
       </c>
     </row>
@@ -3417,7 +3417,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0.963 (0.670-1.383)</t>
+          <t>0.968 (0.674-1.390)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1.006 (0.727-1.394)</t>
+          <t>1.010 (0.730-1.398)</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -3447,7 +3447,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0.858 (0.604-1.218)</t>
+          <t>0.864 (0.609-1.227)</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -3457,7 +3457,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>0.894 (0.710-1.126)</t>
+          <t>0.899 (0.714-1.132)</t>
         </is>
       </c>
     </row>
@@ -3479,7 +3479,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.001 (0.986-1.016)</t>
+          <t>1.000 (0.986-1.015)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -3489,7 +3489,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0.979 (0.394-2.431)</t>
+          <t>0.952 (0.383-2.363)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -3499,7 +3499,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1.032 (0.459-2.319)</t>
+          <t>1.007 (0.448-2.262)</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -3509,7 +3509,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>0.995 (0.989-1.002)</t>
+          <t>0.996 (0.989-1.002)</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -3519,7 +3519,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0.674 (0.314-1.445)</t>
+          <t>0.668 (0.312-1.432)</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -3529,7 +3529,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>0.732 (0.464-1.154)</t>
+          <t>0.736 (0.466-1.160)</t>
         </is>
       </c>
     </row>
@@ -3551,7 +3551,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.999 (0.990-1.007)</t>
+          <t>0.999 (0.990-1.008)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -3561,7 +3561,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0.959 (0.572-1.609)</t>
+          <t>0.975 (0.581-1.636)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -3571,7 +3571,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>0.952 (0.586-1.545)</t>
+          <t>0.965 (0.595-1.567)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -3581,7 +3581,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>0.999 (0.994-1.004)</t>
+          <t>0.999 (0.994-1.005)</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -3591,7 +3591,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0.939 (0.570-1.547)</t>
+          <t>0.954 (0.579-1.572)</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -3601,7 +3601,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>0.950 (0.671-1.345)</t>
+          <t>0.958 (0.677-1.356)</t>
         </is>
       </c>
     </row>
@@ -3623,7 +3623,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.996 (0.982-1.010)</t>
+          <t>0.996 (0.981-1.010)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0.739 (0.296-1.848)</t>
+          <t>0.720 (0.288-1.799)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -3643,7 +3643,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>0.799 (0.358-1.782)</t>
+          <t>0.781 (0.350-1.744)</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -3663,7 +3663,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0.457 (0.213-0.979)</t>
+          <t>0.454 (0.212-0.973)</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -3673,7 +3673,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>0.559 (0.359-0.871)</t>
+          <t>0.563 (0.361-0.878)</t>
         </is>
       </c>
     </row>
@@ -3705,7 +3705,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1.867 (0.489-7.130)</t>
+          <t>1.876 (0.492-7.153)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -3715,7 +3715,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1.898 (0.559-6.449)</t>
+          <t>1.895 (0.559-6.423)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -3725,7 +3725,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>0.991 (0.983-1.000)</t>
+          <t>0.992 (0.984-1.000)</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -3735,7 +3735,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0.776 (0.258-2.333)</t>
+          <t>0.793 (0.264-2.377)</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -3745,7 +3745,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>0.632 (0.333-1.200)</t>
+          <t>0.648 (0.342-1.230)</t>
         </is>
       </c>
     </row>
@@ -3777,7 +3777,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0.923 (0.553-1.541)</t>
+          <t>0.927 (0.555-1.548)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -3787,7 +3787,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>0.976 (0.612-1.555)</t>
+          <t>0.979 (0.614-1.560)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -3797,7 +3797,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>1.002 (0.997-1.006)</t>
+          <t>1.002 (0.998-1.006)</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>1.039 (0.646-1.670)</t>
+          <t>1.044 (0.649-1.678)</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -3817,7 +3817,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>1.059 (0.783-1.432)</t>
+          <t>1.062 (0.786-1.434)</t>
         </is>
       </c>
     </row>
@@ -3839,7 +3839,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1.009 (0.988-1.031)</t>
+          <t>1.008 (0.987-1.029)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -3849,7 +3849,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1.475 (0.405-5.374)</t>
+          <t>1.374 (0.377-5.004)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -3859,7 +3859,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1.464 (0.468-4.584)</t>
+          <t>1.378 (0.440-4.313)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -3879,7 +3879,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>1.348 (0.460-3.954)</t>
+          <t>1.317 (0.450-3.860)</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -3889,7 +3889,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>1.108 (0.603-2.037)</t>
+          <t>1.112 (0.605-2.042)</t>
         </is>
       </c>
     </row>
@@ -3911,7 +3911,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.990 (0.978-1.003)</t>
+          <t>0.991 (0.978-1.003)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -3921,7 +3921,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.574 (0.270-1.223)</t>
+          <t>0.585 (0.275-1.243)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -3931,7 +3931,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>0.568 (0.278-1.159)</t>
+          <t>0.577 (0.283-1.177)</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -3951,7 +3951,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0.673 (0.331-1.371)</t>
+          <t>0.680 (0.334-1.384)</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -3961,7 +3961,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>0.797 (0.491-1.296)</t>
+          <t>0.800 (0.493-1.300)</t>
         </is>
       </c>
     </row>
@@ -3983,7 +3983,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0.999 (0.979-1.019)</t>
+          <t>0.998 (0.978-1.018)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -3993,7 +3993,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.790 (0.218-2.864)</t>
+          <t>0.728 (0.201-2.644)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -4003,7 +4003,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>0.826 (0.268-2.553)</t>
+          <t>0.772 (0.250-2.384)</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -4023,7 +4023,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0.850 (0.297-2.432)</t>
+          <t>0.821 (0.287-2.349)</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -4033,7 +4033,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>0.874 (0.489-1.562)</t>
+          <t>0.870 (0.487-1.555)</t>
         </is>
       </c>
     </row>
@@ -4055,7 +4055,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.995 (0.967-1.023)</t>
+          <t>0.994 (0.966-1.023)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -4065,7 +4065,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>0.601 (0.094-3.829)</t>
+          <t>0.580 (0.091-3.686)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -4075,7 +4075,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>0.572 (0.105-3.109)</t>
+          <t>0.552 (0.102-2.990)</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -4095,7 +4095,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0.784 (0.171-3.600)</t>
+          <t>0.781 (0.171-3.567)</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -4105,7 +4105,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>0.803 (0.337-1.910)</t>
+          <t>0.814 (0.343-1.932)</t>
         </is>
       </c>
     </row>
@@ -4137,7 +4137,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>0.847 (0.715-1.004)</t>
+          <t>0.845 (0.713-1.001)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -4147,7 +4147,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>0.835 (0.713-0.977)</t>
+          <t>0.832 (0.711-0.974)</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0.826 (0.704-0.971)</t>
+          <t>0.826 (0.703-0.971)</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -4199,7 +4199,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1.009 (1.002-1.017)</t>
+          <t>1.009 (1.002-1.016)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -4209,7 +4209,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>1.978 (1.274-3.071)</t>
+          <t>1.936 (1.247-3.008)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -4219,7 +4219,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>1.854 (1.254-2.739)</t>
+          <t>1.820 (1.231-2.690)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -4229,7 +4229,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>1.003 (1.000-1.006)</t>
+          <t>1.003 (1.001-1.006)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -4239,7 +4239,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>1.597 (1.119-2.280)</t>
+          <t>1.599 (1.120-2.282)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -4249,7 +4249,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>1.311 (1.071-1.605)</t>
+          <t>1.322 (1.080-1.618)</t>
         </is>
       </c>
     </row>
@@ -4281,7 +4281,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>0.740 (0.580-0.945)</t>
+          <t>0.739 (0.578-0.943)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -4291,7 +4291,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>0.734 (0.582-0.925)</t>
+          <t>0.732 (0.580-0.922)</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -4311,7 +4311,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0.729 (0.579-0.919)</t>
+          <t>0.728 (0.577-0.917)</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -4321,7 +4321,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>0.786 (0.669-0.922)</t>
+          <t>0.783 (0.667-0.919)</t>
         </is>
       </c>
     </row>
@@ -4343,7 +4343,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1.002 (0.996-1.009)</t>
+          <t>1.002 (0.995-1.009)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -4353,7 +4353,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>1.333 (0.869-2.045)</t>
+          <t>1.287 (0.839-1.976)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -4363,7 +4363,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1.239 (0.854-1.799)</t>
+          <t>1.202 (0.828-1.746)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>1.089 (0.776-1.528)</t>
+          <t>1.077 (0.768-1.512)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -4393,7 +4393,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>0.967 (0.803-1.165)</t>
+          <t>0.968 (0.803-1.166)</t>
         </is>
       </c>
     </row>
@@ -4415,7 +4415,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1.002 (0.993-1.012)</t>
+          <t>1.002 (0.992-1.012)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -4425,7 +4425,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>1.366 (0.718-2.596)</t>
+          <t>1.317 (0.692-2.504)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -4435,7 +4435,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>1.271 (0.705-2.292)</t>
+          <t>1.226 (0.680-2.211)</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0.990 (0.592-1.655)</t>
+          <t>0.985 (0.589-1.645)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -4465,7 +4465,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>0.907 (0.678-1.212)</t>
+          <t>0.913 (0.683-1.219)</t>
         </is>
       </c>
     </row>
@@ -4497,7 +4497,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>0.894 (0.762-1.048)</t>
+          <t>0.897 (0.765-1.052)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -4507,7 +4507,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>0.894 (0.772-1.035)</t>
+          <t>0.897 (0.775-1.038)</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -4527,7 +4527,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0.878 (0.755-1.022)</t>
+          <t>0.882 (0.759-1.026)</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -4537,7 +4537,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>0.889 (0.804-0.983)</t>
+          <t>0.892 (0.807-0.986)</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.002 (0.995-1.009)</t>
+          <t>1.002 (0.995-1.008)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -4569,7 +4569,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.092 (0.719-1.659)</t>
+          <t>1.054 (0.694-1.601)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -4579,7 +4579,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1.112 (0.767-1.613)</t>
+          <t>1.078 (0.743-1.563)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -4599,7 +4599,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1.033 (0.734-1.455)</t>
+          <t>1.021 (0.726-1.438)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -4609,7 +4609,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>0.966 (0.792-1.178)</t>
+          <t>0.970 (0.796-1.183)</t>
         </is>
       </c>
     </row>
@@ -4641,7 +4641,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>0.857 (0.682-1.077)</t>
+          <t>0.866 (0.690-1.088)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -4651,7 +4651,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>0.841 (0.678-1.043)</t>
+          <t>0.849 (0.684-1.053)</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -4671,7 +4671,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0.853 (0.687-1.060)</t>
+          <t>0.860 (0.692-1.068)</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -4681,7 +4681,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>0.872 (0.751-1.014)</t>
+          <t>0.875 (0.753-1.017)</t>
         </is>
       </c>
     </row>
@@ -4703,7 +4703,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>1.000 (0.993-1.006)</t>
+          <t>0.999 (0.993-1.005)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -4713,7 +4713,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>0.949 (0.635-1.418)</t>
+          <t>0.909 (0.608-1.360)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -4723,7 +4723,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>0.967 (0.681-1.372)</t>
+          <t>0.932 (0.657-1.323)</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -4743,7 +4743,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0.877 (0.635-1.212)</t>
+          <t>0.862 (0.624-1.190)</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -4775,7 +4775,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>1.000 (0.990-1.009)</t>
+          <t>0.999 (0.990-1.009)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -4785,7 +4785,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>1.053 (0.577-1.922)</t>
+          <t>1.038 (0.569-1.895)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -4795,7 +4795,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1.007 (0.581-1.746)</t>
+          <t>0.990 (0.571-1.717)</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -4815,7 +4815,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0.904 (0.556-1.470)</t>
+          <t>0.907 (0.559-1.473)</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -4825,7 +4825,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>0.766 (0.580-1.011)</t>
+          <t>0.777 (0.589-1.024)</t>
         </is>
       </c>
     </row>
@@ -4857,7 +4857,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>0.896 (0.665-1.207)</t>
+          <t>0.897 (0.665-1.209)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -4867,7 +4867,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>0.885 (0.673-1.165)</t>
+          <t>0.886 (0.673-1.165)</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -4887,7 +4887,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0.914 (0.691-1.210)</t>
+          <t>0.916 (0.692-1.211)</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -4897,7 +4897,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>0.916 (0.761-1.101)</t>
+          <t>0.917 (0.762-1.102)</t>
         </is>
       </c>
     </row>
@@ -4919,7 +4919,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>0.992 (0.979-1.005)</t>
+          <t>0.992 (0.978-1.005)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -4929,7 +4929,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>0.519 (0.226-1.194)</t>
+          <t>0.509 (0.221-1.171)</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -4939,7 +4939,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>0.582 (0.276-1.226)</t>
+          <t>0.572 (0.272-1.204)</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -4949,7 +4949,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>0.999 (0.993-1.004)</t>
+          <t>0.999 (0.994-1.004)</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -4959,7 +4959,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0.866 (0.443-1.693)</t>
+          <t>0.860 (0.440-1.682)</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -4969,7 +4969,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>0.828 (0.557-1.233)</t>
+          <t>0.831 (0.558-1.236)</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0.997 (0.990-1.005)</t>
+          <t>0.998 (0.990-1.005)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>0.892 (0.579-1.375)</t>
+          <t>0.896 (0.581-1.381)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -5011,7 +5011,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>0.871 (0.578-1.312)</t>
+          <t>0.874 (0.580-1.316)</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -5031,7 +5031,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0.863 (0.574-1.297)</t>
+          <t>0.865 (0.576-1.301)</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -5041,7 +5041,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>0.890 (0.671-1.180)</t>
+          <t>0.891 (0.672-1.181)</t>
         </is>
       </c>
     </row>
@@ -5063,7 +5063,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>0.996 (0.984-1.008)</t>
+          <t>0.996 (0.984-1.007)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -5073,7 +5073,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>0.659 (0.309-1.406)</t>
+          <t>0.644 (0.302-1.372)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -5083,7 +5083,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>0.738 (0.382-1.426)</t>
+          <t>0.723 (0.374-1.397)</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -5103,7 +5103,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>1.027 (0.562-1.875)</t>
+          <t>1.015 (0.556-1.854)</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -5113,7 +5113,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>0.965 (0.693-1.345)</t>
+          <t>0.964 (0.692-1.343)</t>
         </is>
       </c>
     </row>
@@ -5135,7 +5135,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>0.983 (0.965-1.001)</t>
+          <t>0.982 (0.965-1.000)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -5145,7 +5145,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>0.318 (0.095-1.062)</t>
+          <t>0.313 (0.094-1.045)</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -5155,7 +5155,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>0.332 (0.111-0.996)</t>
+          <t>0.327 (0.109-0.980)</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -5165,7 +5165,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>0.997 (0.990-1.003)</t>
+          <t>0.997 (0.990-1.004)</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -5175,7 +5175,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0.676 (0.262-1.745)</t>
+          <t>0.674 (0.261-1.737)</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -5185,7 +5185,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>0.662 (0.386-1.136)</t>
+          <t>0.665 (0.388-1.141)</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>1.067 (0.945-1.205)</t>
+          <t>1.066 (0.944-1.204)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -5227,7 +5227,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1.052 (0.942-1.174)</t>
+          <t>1.051 (0.942-1.174)</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -5247,7 +5247,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>1.076 (0.961-1.206)</t>
+          <t>1.076 (0.961-1.205)</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -5289,7 +5289,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>1.108 (0.785-1.563)</t>
+          <t>1.106 (0.784-1.560)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -5299,7 +5299,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1.065 (0.782-1.449)</t>
+          <t>1.062 (0.781-1.446)</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -5329,7 +5329,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>0.924 (0.786-1.086)</t>
+          <t>0.925 (0.787-1.087)</t>
         </is>
       </c>
     </row>
@@ -5371,7 +5371,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1.063 (0.899-1.256)</t>
+          <t>1.063 (0.899-1.257)</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -5433,7 +5433,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>1.177 (0.852-1.625)</t>
+          <t>1.174 (0.850-1.621)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -5443,7 +5443,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>1.133 (0.855-1.502)</t>
+          <t>1.131 (0.853-1.498)</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -5473,7 +5473,7 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>0.962 (0.836-1.107)</t>
+          <t>0.963 (0.837-1.108)</t>
         </is>
       </c>
     </row>
@@ -5505,7 +5505,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>1.566 (0.943-2.601)</t>
+          <t>1.564 (0.942-2.597)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -5515,7 +5515,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>1.471 (0.926-2.338)</t>
+          <t>1.469 (0.924-2.334)</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -5535,7 +5535,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>1.627 (1.096-2.416)</t>
+          <t>1.627 (1.096-2.417)</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -5545,7 +5545,7 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>0.996 (0.798-1.242)</t>
+          <t>0.998 (0.800-1.244)</t>
         </is>
       </c>
     </row>

</xml_diff>